<commit_message>
validation & reconciliation checks in intermediate layer
</commit_message>
<xml_diff>
--- a/data_pipeline/ldf_selection_table.xlsx
+++ b/data_pipeline/ldf_selection_table.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\internship\airflow\dbt_project\data_pipeline\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E81EC909-405A-4214-8F9B-E9AD7DA66B03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86C0BA0E-A9F8-4474-8AB5-2E139D610006}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{F28D853A-AEE6-41FA-B749-E7364606C53D}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="26">
   <si>
     <t>segmentation_version</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -124,6 +124,10 @@
   </si>
   <si>
     <t>claim_count</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>paid</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -488,7 +492,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1841F34B-EA64-406F-BC03-5231868C93CA}">
-  <dimension ref="A1:K18"/>
+  <dimension ref="A1:K33"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
@@ -1067,6 +1071,453 @@
         <v>19</v>
       </c>
     </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>10</v>
+      </c>
+      <c r="B19" t="s">
+        <v>24</v>
+      </c>
+      <c r="C19" t="s">
+        <v>20</v>
+      </c>
+      <c r="D19" t="s">
+        <v>20</v>
+      </c>
+      <c r="E19" t="s">
+        <v>20</v>
+      </c>
+      <c r="F19">
+        <v>5</v>
+      </c>
+      <c r="G19">
+        <v>1</v>
+      </c>
+      <c r="H19" t="s">
+        <v>16</v>
+      </c>
+      <c r="K19" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>10</v>
+      </c>
+      <c r="B20" t="s">
+        <v>24</v>
+      </c>
+      <c r="C20" t="s">
+        <v>20</v>
+      </c>
+      <c r="D20" t="s">
+        <v>20</v>
+      </c>
+      <c r="E20" t="s">
+        <v>20</v>
+      </c>
+      <c r="F20">
+        <v>6</v>
+      </c>
+      <c r="G20">
+        <v>1</v>
+      </c>
+      <c r="H20" t="s">
+        <v>16</v>
+      </c>
+      <c r="K20" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>10</v>
+      </c>
+      <c r="B21" t="s">
+        <v>24</v>
+      </c>
+      <c r="C21" t="s">
+        <v>20</v>
+      </c>
+      <c r="D21" t="s">
+        <v>20</v>
+      </c>
+      <c r="E21" t="s">
+        <v>20</v>
+      </c>
+      <c r="F21">
+        <v>7</v>
+      </c>
+      <c r="G21">
+        <v>1</v>
+      </c>
+      <c r="H21" t="s">
+        <v>16</v>
+      </c>
+      <c r="K21" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>10</v>
+      </c>
+      <c r="B22" t="s">
+        <v>24</v>
+      </c>
+      <c r="C22" t="s">
+        <v>20</v>
+      </c>
+      <c r="D22" t="s">
+        <v>20</v>
+      </c>
+      <c r="E22" t="s">
+        <v>20</v>
+      </c>
+      <c r="F22">
+        <v>8</v>
+      </c>
+      <c r="G22">
+        <v>1</v>
+      </c>
+      <c r="H22" t="s">
+        <v>16</v>
+      </c>
+      <c r="K22" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>10</v>
+      </c>
+      <c r="B23" t="s">
+        <v>24</v>
+      </c>
+      <c r="C23" t="s">
+        <v>20</v>
+      </c>
+      <c r="D23" t="s">
+        <v>20</v>
+      </c>
+      <c r="E23" t="s">
+        <v>20</v>
+      </c>
+      <c r="F23">
+        <v>9</v>
+      </c>
+      <c r="G23">
+        <v>1</v>
+      </c>
+      <c r="H23" t="s">
+        <v>16</v>
+      </c>
+      <c r="K23" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>10</v>
+      </c>
+      <c r="B24" t="s">
+        <v>25</v>
+      </c>
+      <c r="C24" t="s">
+        <v>20</v>
+      </c>
+      <c r="D24" t="s">
+        <v>20</v>
+      </c>
+      <c r="E24" t="s">
+        <v>20</v>
+      </c>
+      <c r="F24">
+        <v>0</v>
+      </c>
+      <c r="G24">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="H24" t="s">
+        <v>12</v>
+      </c>
+      <c r="I24">
+        <v>2020</v>
+      </c>
+      <c r="J24">
+        <v>2022</v>
+      </c>
+      <c r="K24" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>10</v>
+      </c>
+      <c r="B25" t="s">
+        <v>25</v>
+      </c>
+      <c r="C25" t="s">
+        <v>20</v>
+      </c>
+      <c r="D25" t="s">
+        <v>20</v>
+      </c>
+      <c r="E25" t="s">
+        <v>20</v>
+      </c>
+      <c r="F25">
+        <v>1</v>
+      </c>
+      <c r="G25">
+        <v>1.24</v>
+      </c>
+      <c r="H25" t="s">
+        <v>17</v>
+      </c>
+      <c r="I25">
+        <v>2019</v>
+      </c>
+      <c r="J25">
+        <v>2021</v>
+      </c>
+      <c r="K25" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>10</v>
+      </c>
+      <c r="B26" t="s">
+        <v>25</v>
+      </c>
+      <c r="C26" t="s">
+        <v>20</v>
+      </c>
+      <c r="D26" t="s">
+        <v>20</v>
+      </c>
+      <c r="E26" t="s">
+        <v>20</v>
+      </c>
+      <c r="F26">
+        <v>2</v>
+      </c>
+      <c r="G26">
+        <v>1.01</v>
+      </c>
+      <c r="H26" t="s">
+        <v>16</v>
+      </c>
+      <c r="K26" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>10</v>
+      </c>
+      <c r="B27" t="s">
+        <v>25</v>
+      </c>
+      <c r="C27" t="s">
+        <v>20</v>
+      </c>
+      <c r="D27" t="s">
+        <v>20</v>
+      </c>
+      <c r="E27" t="s">
+        <v>20</v>
+      </c>
+      <c r="F27">
+        <v>3</v>
+      </c>
+      <c r="G27">
+        <v>1</v>
+      </c>
+      <c r="H27" t="s">
+        <v>16</v>
+      </c>
+      <c r="K27" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>10</v>
+      </c>
+      <c r="B28" t="s">
+        <v>25</v>
+      </c>
+      <c r="C28" t="s">
+        <v>20</v>
+      </c>
+      <c r="D28" t="s">
+        <v>20</v>
+      </c>
+      <c r="E28" t="s">
+        <v>20</v>
+      </c>
+      <c r="F28">
+        <v>4</v>
+      </c>
+      <c r="G28">
+        <v>1</v>
+      </c>
+      <c r="H28" t="s">
+        <v>16</v>
+      </c>
+      <c r="K28" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>10</v>
+      </c>
+      <c r="B29" t="s">
+        <v>25</v>
+      </c>
+      <c r="C29" t="s">
+        <v>20</v>
+      </c>
+      <c r="D29" t="s">
+        <v>20</v>
+      </c>
+      <c r="E29" t="s">
+        <v>20</v>
+      </c>
+      <c r="F29">
+        <v>5</v>
+      </c>
+      <c r="G29">
+        <v>1</v>
+      </c>
+      <c r="H29" t="s">
+        <v>16</v>
+      </c>
+      <c r="K29" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>10</v>
+      </c>
+      <c r="B30" t="s">
+        <v>25</v>
+      </c>
+      <c r="C30" t="s">
+        <v>20</v>
+      </c>
+      <c r="D30" t="s">
+        <v>20</v>
+      </c>
+      <c r="E30" t="s">
+        <v>20</v>
+      </c>
+      <c r="F30">
+        <v>6</v>
+      </c>
+      <c r="G30">
+        <v>1</v>
+      </c>
+      <c r="H30" t="s">
+        <v>16</v>
+      </c>
+      <c r="K30" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>10</v>
+      </c>
+      <c r="B31" t="s">
+        <v>25</v>
+      </c>
+      <c r="C31" t="s">
+        <v>20</v>
+      </c>
+      <c r="D31" t="s">
+        <v>20</v>
+      </c>
+      <c r="E31" t="s">
+        <v>20</v>
+      </c>
+      <c r="F31">
+        <v>7</v>
+      </c>
+      <c r="G31">
+        <v>1</v>
+      </c>
+      <c r="H31" t="s">
+        <v>16</v>
+      </c>
+      <c r="K31" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>10</v>
+      </c>
+      <c r="B32" t="s">
+        <v>25</v>
+      </c>
+      <c r="C32" t="s">
+        <v>20</v>
+      </c>
+      <c r="D32" t="s">
+        <v>20</v>
+      </c>
+      <c r="E32" t="s">
+        <v>20</v>
+      </c>
+      <c r="F32">
+        <v>8</v>
+      </c>
+      <c r="G32">
+        <v>1</v>
+      </c>
+      <c r="H32" t="s">
+        <v>16</v>
+      </c>
+      <c r="K32" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>10</v>
+      </c>
+      <c r="B33" t="s">
+        <v>25</v>
+      </c>
+      <c r="C33" t="s">
+        <v>20</v>
+      </c>
+      <c r="D33" t="s">
+        <v>20</v>
+      </c>
+      <c r="E33" t="s">
+        <v>20</v>
+      </c>
+      <c r="F33">
+        <v>9</v>
+      </c>
+      <c r="G33">
+        <v>1</v>
+      </c>
+      <c r="H33" t="s">
+        <v>16</v>
+      </c>
+      <c r="K33" t="s">
+        <v>19</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
intermediate validation & reconciliation & partial governance
</commit_message>
<xml_diff>
--- a/data_pipeline/ldf_selection_table.xlsx
+++ b/data_pipeline/ldf_selection_table.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\internship\airflow\dbt_project\data_pipeline\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86C0BA0E-A9F8-4474-8AB5-2E139D610006}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35781E97-D5A4-49DA-9B57-443DDFE60FD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{F28D853A-AEE6-41FA-B749-E7364606C53D}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="28">
   <si>
     <t>segmentation_version</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -83,14 +83,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>ay_from</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>ay_to</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>other</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -128,6 +120,21 @@
   </si>
   <si>
     <t>paid</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>weighted</t>
+  </si>
+  <si>
+    <t>oooooooo</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>flat</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>guess</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -492,15 +499,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1841F34B-EA64-406F-BC03-5231868C93CA}">
-  <dimension ref="A1:K33"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
@@ -512,7 +519,7 @@
         <v>3</v>
       </c>
       <c r="F1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="G1" t="s">
         <v>4</v>
@@ -521,21 +528,15 @@
         <v>11</v>
       </c>
       <c r="I1" t="s">
-        <v>14</v>
-      </c>
-      <c r="J1" t="s">
-        <v>15</v>
-      </c>
-      <c r="K1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C2" t="s">
         <v>6</v>
@@ -544,7 +545,7 @@
         <v>7</v>
       </c>
       <c r="E2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -553,18 +554,18 @@
         <v>1.4</v>
       </c>
       <c r="H2" t="s">
-        <v>17</v>
-      </c>
-      <c r="K2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+        <v>15</v>
+      </c>
+      <c r="I2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>5</v>
       </c>
       <c r="B3" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C3" t="s">
         <v>6</v>
@@ -573,7 +574,7 @@
         <v>7</v>
       </c>
       <c r="E3" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F3">
         <v>1</v>
@@ -584,22 +585,16 @@
       <c r="H3" t="s">
         <v>12</v>
       </c>
-      <c r="I3">
-        <v>2019</v>
-      </c>
-      <c r="J3">
-        <v>2023</v>
-      </c>
-      <c r="K3" t="s">
+      <c r="I3" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>5</v>
       </c>
       <c r="B4" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C4" t="s">
         <v>6</v>
@@ -608,7 +603,7 @@
         <v>7</v>
       </c>
       <c r="E4" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F4">
         <v>2</v>
@@ -619,22 +614,16 @@
       <c r="H4" t="s">
         <v>13</v>
       </c>
-      <c r="I4">
-        <v>2019</v>
-      </c>
-      <c r="J4">
-        <v>2023</v>
-      </c>
-      <c r="K4" t="s">
+      <c r="I4" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C5" t="s">
         <v>6</v>
@@ -643,7 +632,7 @@
         <v>8</v>
       </c>
       <c r="E5" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F5">
         <v>0</v>
@@ -652,18 +641,18 @@
         <v>1.5</v>
       </c>
       <c r="H5" t="s">
-        <v>17</v>
-      </c>
-      <c r="K5" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+        <v>15</v>
+      </c>
+      <c r="I5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C6" t="s">
         <v>6</v>
@@ -672,7 +661,7 @@
         <v>8</v>
       </c>
       <c r="E6" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F6">
         <v>1</v>
@@ -683,31 +672,25 @@
       <c r="H6" t="s">
         <v>12</v>
       </c>
-      <c r="I6">
-        <v>2019</v>
-      </c>
-      <c r="J6">
-        <v>2023</v>
-      </c>
-      <c r="K6" t="s">
+      <c r="I6" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
       <c r="B7" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C7" t="s">
         <v>6</v>
       </c>
       <c r="D7" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E7" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F7">
         <v>0</v>
@@ -718,159 +701,141 @@
       <c r="H7" t="s">
         <v>13</v>
       </c>
-      <c r="I7">
-        <v>2019</v>
-      </c>
-      <c r="J7">
-        <v>2023</v>
-      </c>
-      <c r="K7" t="s">
+      <c r="I7" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>9</v>
       </c>
       <c r="B8" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C8" t="s">
         <v>6</v>
       </c>
       <c r="D8" t="s">
+        <v>18</v>
+      </c>
+      <c r="E8" t="s">
+        <v>18</v>
+      </c>
+      <c r="F8">
+        <v>1</v>
+      </c>
+      <c r="G8">
+        <v>1.05</v>
+      </c>
+      <c r="H8" t="s">
+        <v>14</v>
+      </c>
+      <c r="I8" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" t="s">
         <v>20</v>
       </c>
-      <c r="E8" t="s">
-        <v>20</v>
-      </c>
-      <c r="F8">
-        <v>1</v>
-      </c>
-      <c r="G8">
-        <v>1.25</v>
-      </c>
-      <c r="H8" t="s">
-        <v>17</v>
-      </c>
-      <c r="K8" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>10</v>
-      </c>
-      <c r="B9" t="s">
-        <v>22</v>
-      </c>
       <c r="C9" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D9" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E9" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F9">
         <v>0</v>
       </c>
       <c r="G9">
-        <v>1.3</v>
+        <v>1.05</v>
       </c>
       <c r="H9" t="s">
-        <v>12</v>
-      </c>
-      <c r="I9">
-        <v>2020</v>
-      </c>
-      <c r="J9">
-        <v>2022</v>
-      </c>
-      <c r="K9" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+        <v>14</v>
+      </c>
+      <c r="I9" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>10</v>
       </c>
       <c r="B10" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D10" t="s">
+        <v>18</v>
+      </c>
+      <c r="E10" t="s">
+        <v>18</v>
+      </c>
+      <c r="F10">
+        <v>1</v>
+      </c>
+      <c r="G10">
+        <v>1</v>
+      </c>
+      <c r="H10" t="s">
+        <v>14</v>
+      </c>
+      <c r="I10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
         <v>20</v>
       </c>
-      <c r="D10" t="s">
-        <v>20</v>
-      </c>
-      <c r="E10" t="s">
-        <v>20</v>
-      </c>
-      <c r="F10">
-        <v>1</v>
-      </c>
-      <c r="G10">
-        <v>1.2</v>
-      </c>
-      <c r="H10" t="s">
-        <v>17</v>
-      </c>
-      <c r="I10">
-        <v>2019</v>
-      </c>
-      <c r="J10">
-        <v>2021</v>
-      </c>
-      <c r="K10" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>10</v>
-      </c>
-      <c r="B11" t="s">
-        <v>22</v>
-      </c>
       <c r="C11" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D11" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E11" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F11">
         <v>2</v>
       </c>
       <c r="G11">
-        <v>1.1000000000000001</v>
+        <v>1</v>
       </c>
       <c r="H11" t="s">
-        <v>16</v>
-      </c>
-      <c r="K11" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+        <v>14</v>
+      </c>
+      <c r="I11" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C12" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D12" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E12" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F12">
         <v>3</v>
@@ -879,27 +844,27 @@
         <v>1</v>
       </c>
       <c r="H12" t="s">
-        <v>16</v>
-      </c>
-      <c r="K12" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+        <v>14</v>
+      </c>
+      <c r="I12" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>10</v>
       </c>
       <c r="B13" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C13" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D13" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E13" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F13">
         <v>4</v>
@@ -908,27 +873,27 @@
         <v>1</v>
       </c>
       <c r="H13" t="s">
-        <v>16</v>
-      </c>
-      <c r="K13" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+        <v>14</v>
+      </c>
+      <c r="I13" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>10</v>
       </c>
       <c r="B14" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C14" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D14" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E14" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F14">
         <v>0</v>
@@ -939,31 +904,25 @@
       <c r="H14" t="s">
         <v>12</v>
       </c>
-      <c r="I14">
-        <v>2020</v>
-      </c>
-      <c r="J14">
-        <v>2022</v>
-      </c>
-      <c r="K14" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="I14" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>10</v>
       </c>
       <c r="B15" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C15" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D15" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E15" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F15">
         <v>1</v>
@@ -972,33 +931,27 @@
         <v>1.2</v>
       </c>
       <c r="H15" t="s">
-        <v>17</v>
-      </c>
-      <c r="I15">
-        <v>2019</v>
-      </c>
-      <c r="J15">
-        <v>2021</v>
-      </c>
-      <c r="K15" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+        <v>15</v>
+      </c>
+      <c r="I15" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>10</v>
       </c>
       <c r="B16" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C16" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D16" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E16" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F16">
         <v>2</v>
@@ -1007,27 +960,27 @@
         <v>1</v>
       </c>
       <c r="H16" t="s">
-        <v>16</v>
-      </c>
-      <c r="K16" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+        <v>14</v>
+      </c>
+      <c r="I16" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>10</v>
       </c>
       <c r="B17" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C17" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D17" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E17" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F17">
         <v>3</v>
@@ -1036,27 +989,27 @@
         <v>1</v>
       </c>
       <c r="H17" t="s">
-        <v>16</v>
-      </c>
-      <c r="K17" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+        <v>14</v>
+      </c>
+      <c r="I17" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>10</v>
       </c>
       <c r="B18" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C18" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D18" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E18" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F18">
         <v>4</v>
@@ -1065,457 +1018,155 @@
         <v>1</v>
       </c>
       <c r="H18" t="s">
-        <v>16</v>
-      </c>
-      <c r="K18" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+        <v>14</v>
+      </c>
+      <c r="I18" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>10</v>
       </c>
       <c r="B19" t="s">
+        <v>23</v>
+      </c>
+      <c r="C19" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19" t="s">
+        <v>18</v>
+      </c>
+      <c r="E19" t="s">
+        <v>18</v>
+      </c>
+      <c r="F19">
+        <v>0</v>
+      </c>
+      <c r="G19">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="H19" t="s">
+        <v>15</v>
+      </c>
+      <c r="I19" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>10</v>
+      </c>
+      <c r="B20" t="s">
+        <v>23</v>
+      </c>
+      <c r="C20" t="s">
+        <v>18</v>
+      </c>
+      <c r="D20" t="s">
+        <v>18</v>
+      </c>
+      <c r="E20" t="s">
+        <v>18</v>
+      </c>
+      <c r="F20">
+        <v>1</v>
+      </c>
+      <c r="G20">
+        <v>1.24</v>
+      </c>
+      <c r="H20" t="s">
         <v>24</v>
       </c>
-      <c r="C19" t="s">
-        <v>20</v>
-      </c>
-      <c r="D19" t="s">
-        <v>20</v>
-      </c>
-      <c r="E19" t="s">
-        <v>20</v>
-      </c>
-      <c r="F19">
-        <v>5</v>
-      </c>
-      <c r="G19">
-        <v>1</v>
-      </c>
-      <c r="H19" t="s">
-        <v>16</v>
-      </c>
-      <c r="K19" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
-        <v>10</v>
-      </c>
-      <c r="B20" t="s">
-        <v>24</v>
-      </c>
-      <c r="C20" t="s">
-        <v>20</v>
-      </c>
-      <c r="D20" t="s">
-        <v>20</v>
-      </c>
-      <c r="E20" t="s">
-        <v>20</v>
-      </c>
-      <c r="F20">
-        <v>6</v>
-      </c>
-      <c r="G20">
-        <v>1</v>
-      </c>
-      <c r="H20" t="s">
-        <v>16</v>
-      </c>
-      <c r="K20" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="I20" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>10</v>
       </c>
       <c r="B21" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C21" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D21" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E21" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F21">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="G21">
-        <v>1</v>
+        <v>1.01</v>
       </c>
       <c r="H21" t="s">
-        <v>16</v>
-      </c>
-      <c r="K21" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
+        <v>14</v>
+      </c>
+      <c r="I21" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>10</v>
       </c>
       <c r="B22" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C22" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D22" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E22" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F22">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G22">
         <v>1</v>
       </c>
       <c r="H22" t="s">
-        <v>16</v>
-      </c>
-      <c r="K22" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+        <v>14</v>
+      </c>
+      <c r="I22" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>10</v>
       </c>
       <c r="B23" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C23" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D23" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E23" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F23">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="G23">
         <v>1</v>
       </c>
       <c r="H23" t="s">
-        <v>16</v>
-      </c>
-      <c r="K23" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A24" t="s">
-        <v>10</v>
-      </c>
-      <c r="B24" t="s">
-        <v>25</v>
-      </c>
-      <c r="C24" t="s">
-        <v>20</v>
-      </c>
-      <c r="D24" t="s">
-        <v>20</v>
-      </c>
-      <c r="E24" t="s">
-        <v>20</v>
-      </c>
-      <c r="F24">
-        <v>0</v>
-      </c>
-      <c r="G24">
-        <v>2.2999999999999998</v>
-      </c>
-      <c r="H24" t="s">
-        <v>12</v>
-      </c>
-      <c r="I24">
-        <v>2020</v>
-      </c>
-      <c r="J24">
-        <v>2022</v>
-      </c>
-      <c r="K24" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
-        <v>10</v>
-      </c>
-      <c r="B25" t="s">
-        <v>25</v>
-      </c>
-      <c r="C25" t="s">
-        <v>20</v>
-      </c>
-      <c r="D25" t="s">
-        <v>20</v>
-      </c>
-      <c r="E25" t="s">
-        <v>20</v>
-      </c>
-      <c r="F25">
-        <v>1</v>
-      </c>
-      <c r="G25">
-        <v>1.24</v>
-      </c>
-      <c r="H25" t="s">
+        <v>14</v>
+      </c>
+      <c r="I23" t="s">
         <v>17</v>
-      </c>
-      <c r="I25">
-        <v>2019</v>
-      </c>
-      <c r="J25">
-        <v>2021</v>
-      </c>
-      <c r="K25" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A26" t="s">
-        <v>10</v>
-      </c>
-      <c r="B26" t="s">
-        <v>25</v>
-      </c>
-      <c r="C26" t="s">
-        <v>20</v>
-      </c>
-      <c r="D26" t="s">
-        <v>20</v>
-      </c>
-      <c r="E26" t="s">
-        <v>20</v>
-      </c>
-      <c r="F26">
-        <v>2</v>
-      </c>
-      <c r="G26">
-        <v>1.01</v>
-      </c>
-      <c r="H26" t="s">
-        <v>16</v>
-      </c>
-      <c r="K26" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
-        <v>10</v>
-      </c>
-      <c r="B27" t="s">
-        <v>25</v>
-      </c>
-      <c r="C27" t="s">
-        <v>20</v>
-      </c>
-      <c r="D27" t="s">
-        <v>20</v>
-      </c>
-      <c r="E27" t="s">
-        <v>20</v>
-      </c>
-      <c r="F27">
-        <v>3</v>
-      </c>
-      <c r="G27">
-        <v>1</v>
-      </c>
-      <c r="H27" t="s">
-        <v>16</v>
-      </c>
-      <c r="K27" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A28" t="s">
-        <v>10</v>
-      </c>
-      <c r="B28" t="s">
-        <v>25</v>
-      </c>
-      <c r="C28" t="s">
-        <v>20</v>
-      </c>
-      <c r="D28" t="s">
-        <v>20</v>
-      </c>
-      <c r="E28" t="s">
-        <v>20</v>
-      </c>
-      <c r="F28">
-        <v>4</v>
-      </c>
-      <c r="G28">
-        <v>1</v>
-      </c>
-      <c r="H28" t="s">
-        <v>16</v>
-      </c>
-      <c r="K28" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A29" t="s">
-        <v>10</v>
-      </c>
-      <c r="B29" t="s">
-        <v>25</v>
-      </c>
-      <c r="C29" t="s">
-        <v>20</v>
-      </c>
-      <c r="D29" t="s">
-        <v>20</v>
-      </c>
-      <c r="E29" t="s">
-        <v>20</v>
-      </c>
-      <c r="F29">
-        <v>5</v>
-      </c>
-      <c r="G29">
-        <v>1</v>
-      </c>
-      <c r="H29" t="s">
-        <v>16</v>
-      </c>
-      <c r="K29" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A30" t="s">
-        <v>10</v>
-      </c>
-      <c r="B30" t="s">
-        <v>25</v>
-      </c>
-      <c r="C30" t="s">
-        <v>20</v>
-      </c>
-      <c r="D30" t="s">
-        <v>20</v>
-      </c>
-      <c r="E30" t="s">
-        <v>20</v>
-      </c>
-      <c r="F30">
-        <v>6</v>
-      </c>
-      <c r="G30">
-        <v>1</v>
-      </c>
-      <c r="H30" t="s">
-        <v>16</v>
-      </c>
-      <c r="K30" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A31" t="s">
-        <v>10</v>
-      </c>
-      <c r="B31" t="s">
-        <v>25</v>
-      </c>
-      <c r="C31" t="s">
-        <v>20</v>
-      </c>
-      <c r="D31" t="s">
-        <v>20</v>
-      </c>
-      <c r="E31" t="s">
-        <v>20</v>
-      </c>
-      <c r="F31">
-        <v>7</v>
-      </c>
-      <c r="G31">
-        <v>1</v>
-      </c>
-      <c r="H31" t="s">
-        <v>16</v>
-      </c>
-      <c r="K31" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A32" t="s">
-        <v>10</v>
-      </c>
-      <c r="B32" t="s">
-        <v>25</v>
-      </c>
-      <c r="C32" t="s">
-        <v>20</v>
-      </c>
-      <c r="D32" t="s">
-        <v>20</v>
-      </c>
-      <c r="E32" t="s">
-        <v>20</v>
-      </c>
-      <c r="F32">
-        <v>8</v>
-      </c>
-      <c r="G32">
-        <v>1</v>
-      </c>
-      <c r="H32" t="s">
-        <v>16</v>
-      </c>
-      <c r="K32" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A33" t="s">
-        <v>10</v>
-      </c>
-      <c r="B33" t="s">
-        <v>25</v>
-      </c>
-      <c r="C33" t="s">
-        <v>20</v>
-      </c>
-      <c r="D33" t="s">
-        <v>20</v>
-      </c>
-      <c r="E33" t="s">
-        <v>20</v>
-      </c>
-      <c r="F33">
-        <v>9</v>
-      </c>
-      <c r="G33">
-        <v>1</v>
-      </c>
-      <c r="H33" t="s">
-        <v>16</v>
-      </c>
-      <c r="K33" t="s">
-        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>